<commit_message>
them procedure va sua class DatabaseConnector
</commit_message>
<xml_diff>
--- a/Database/DatabaseTasks.xlsx
+++ b/Database/DatabaseTasks.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25924"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -15,10 +15,21 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -27,110 +38,110 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
+    <t>Ngày thực hiện 18/11/2022</t>
+  </si>
+  <si>
     <t>Task CSDL</t>
   </si>
   <si>
+    <t>Công việc</t>
+  </si>
+  <si>
+    <t>Dự kiến thoàn thành</t>
+  </si>
+  <si>
+    <t>Trạng thái</t>
+  </si>
+  <si>
+    <t>Tên file yêu cầu</t>
+  </si>
+  <si>
+    <t>Người thực hiện</t>
+  </si>
+  <si>
+    <t>Ghi chú</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mô tả bài toán: mục đích, yêu cầu, quy trình xử lý bên trong hệ thống. </t>
+  </si>
+  <si>
+    <t>PhanTichNghiepVu.docx</t>
+  </si>
+  <si>
     <t xml:space="preserve">Đưa ra mô hình liên kết thực thể (ER): Mô tả tập thực thể, thuộc tính, mối quan hệ. </t>
   </si>
   <si>
-    <t xml:space="preserve">Mô tả bài toán: mục đích, yêu cầu, quy trình xử lý bên trong hệ thống. </t>
+    <t>ERdiagram.jpg</t>
+  </si>
+  <si>
+    <t>Chuyển lược đồ ER sang mô hình quan hệ tối thiểu chuẩn 3NF</t>
+  </si>
+  <si>
+    <t>RelationalDataModel.docx</t>
   </si>
   <si>
     <t xml:space="preserve">Thiết kế (cài đặt CSDL) các bảng dữ liệu. Mô tả chính xác các mối quan hệ, ràng buộc toàn vẹn, khóa chính, khóa ngoại... </t>
   </si>
   <si>
+    <t>BookStoreManagement.sql</t>
+  </si>
+  <si>
+    <t>Vẽ diagram table sau khi đã chuẩn hóa 3NF</t>
+  </si>
+  <si>
+    <t>RelationalDiagram.jpg</t>
+  </si>
+  <si>
     <t xml:space="preserve">Làm data, mỗi bảng 10 bản ghi, các bảng có khóa ngoại lập ít nhất 20 bản ghi  </t>
   </si>
   <si>
+    <t>Data.xlsx</t>
+  </si>
+  <si>
+    <t>mỗi sheet trong file excel là dữ liệu của 1 bảng</t>
+  </si>
+  <si>
+    <t>Viết và chạy truy vấn trên csdl đã tạo, tối thiểu 4 truy vấn mỗi bảng, có ít nhất 2 truy vấn sử dụng group by, having, limit, sort…</t>
+  </si>
+  <si>
+    <t>Query&lt;Tên bảng 1_tên bảng 2_...&gt;n.sql</t>
+  </si>
+  <si>
+    <t>mỗi câu truy vấn 1 file, tên bảng là các bảng sử dụng trong câu truy vấn, viết bằng CamelCase, mỗi bảng cách nhau bằng '_'  cuối file đặt thêm số n = 1,2,3,... để phân biệt các câu truy vấn với nhau sau đó cho vào 1 folder tên là Query</t>
+  </si>
+  <si>
+    <t>Thực hiện viết trigger cho csdl</t>
+  </si>
+  <si>
+    <t>Trigger.sql</t>
+  </si>
+  <si>
+    <t>viết tất cả trigger vào 1 file</t>
+  </si>
+  <si>
     <t>Thực hiện viết procedure cho csdl</t>
   </si>
   <si>
-    <t>Thực hiện viết trigger cho csdl</t>
-  </si>
-  <si>
-    <t>Người thực hiện</t>
-  </si>
-  <si>
-    <t>Tên file yêu cầu</t>
-  </si>
-  <si>
-    <t>Công việc</t>
-  </si>
-  <si>
-    <t>Ghi chú</t>
-  </si>
-  <si>
-    <t>Ngày thực hiện 18/11/2022</t>
-  </si>
-  <si>
-    <t>PhanTichNghiepVu.docx</t>
-  </si>
-  <si>
-    <t>ERdiagram.jpg</t>
-  </si>
-  <si>
-    <t>Dự kiến thoàn thành</t>
-  </si>
-  <si>
-    <t>Trạng thái</t>
-  </si>
-  <si>
-    <t>Chuyển lược đồ ER sang mô hình quan hệ tối thiểu chuẩn 3NF</t>
-  </si>
-  <si>
-    <t>Vẽ diagram table sau khi đã chuẩn hóa 3NF</t>
-  </si>
-  <si>
-    <t>Viết và chạy truy vấn trên csdl đã tạo, tối thiểu 4 truy vấn mỗi bảng, có ít nhất 2 truy vấn sử dụng group by, having, limit, sort…</t>
+    <t>Procedure.sql</t>
+  </si>
+  <si>
+    <t>viết tất cả procedure vào 1 file</t>
   </si>
   <si>
     <t>Viết test các trigger, procedure</t>
   </si>
   <si>
-    <t>RelationalDataModel.docx</t>
-  </si>
-  <si>
-    <t>RelationalDiagram.jpg</t>
-  </si>
-  <si>
-    <t>Data.xlsx</t>
-  </si>
-  <si>
-    <t>mỗi sheet trong file excel là dữ liệu của 1 bảng</t>
-  </si>
-  <si>
-    <t>viết tất cả trigger vào 1 file</t>
-  </si>
-  <si>
-    <t>Query&lt;Tên bảng 1_tên bảng 2_...&gt;n.sql</t>
-  </si>
-  <si>
-    <t>viết tất cả procedure vào 1 file</t>
-  </si>
-  <si>
-    <t>Trigger.sql</t>
-  </si>
-  <si>
-    <t>Procedure.sql</t>
-  </si>
-  <si>
     <t>Trigger/Procedure&lt;Tên Trigger hoặc Procedure&gt;Test.sql</t>
   </si>
   <si>
-    <t>mỗi câu truy vấn 1 file, tên bảng là các bảng sử dụng trong câu truy vấn, viết bằng CamelCase, mỗi bảng cách nhau bằng '_'  cuối file đặt thêm số n = 1,2,3,... để phân biệt các câu truy vấn với nhau sau đó cho vào 1 folder tên là Query</t>
-  </si>
-  <si>
     <t>mỗi trigger hoặc 1 procedure viết 1 test sau đó lưu vào một Folder.</t>
-  </si>
-  <si>
-    <t>BookStoreManagement.sql</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1274,7 +1285,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:H13"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="5.75" customWidth="1"/>
     <col min="2" max="2" width="9.125" customWidth="1"/>
@@ -1286,166 +1297,166 @@
     <col min="8" max="8" width="43" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:8" ht="15" thickBot="1">
       <c r="C2" t="s">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:8" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:8" ht="27" customHeight="1">
       <c r="B3" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="H3" s="4" t="s">
-        <v>10</v>
-      </c>
     </row>
-    <row r="4" spans="2:8" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:8" ht="31.5" customHeight="1">
       <c r="B4" s="8">
         <v>1</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
       <c r="F4" s="10" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="G4" s="9"/>
       <c r="H4" s="11"/>
     </row>
-    <row r="5" spans="2:8" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:8" ht="31.5" customHeight="1">
       <c r="B5" s="12">
         <v>2</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D5" s="13"/>
       <c r="E5" s="13"/>
       <c r="F5" s="14" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G5" s="13"/>
       <c r="H5" s="15"/>
     </row>
-    <row r="6" spans="2:8" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:8" ht="31.5" customHeight="1">
       <c r="B6" s="12">
         <v>3</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D6" s="13"/>
       <c r="E6" s="13"/>
       <c r="F6" s="14" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="G6" s="13"/>
       <c r="H6" s="15"/>
     </row>
-    <row r="7" spans="2:8" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:8" ht="31.5" customHeight="1">
       <c r="B7" s="12">
         <v>4</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="D7" s="13"/>
       <c r="E7" s="13"/>
       <c r="F7" s="14" t="s">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="G7" s="13"/>
       <c r="H7" s="15"/>
     </row>
-    <row r="8" spans="2:8" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:8" ht="31.5" customHeight="1">
       <c r="B8" s="12">
         <v>5</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D8" s="13"/>
       <c r="E8" s="13"/>
       <c r="F8" s="14" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="G8" s="13"/>
       <c r="H8" s="15"/>
     </row>
-    <row r="9" spans="2:8" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:8" ht="31.5" customHeight="1">
       <c r="B9" s="12">
         <v>6</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="D9" s="13"/>
       <c r="E9" s="13"/>
       <c r="F9" s="14" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="G9" s="13"/>
       <c r="H9" s="15" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
-    <row r="10" spans="2:8" ht="105" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:8" ht="105" customHeight="1">
       <c r="B10" s="12">
         <v>7</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D10" s="13"/>
       <c r="E10" s="13"/>
       <c r="F10" s="14" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="G10" s="13"/>
       <c r="H10" s="15" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
     </row>
-    <row r="11" spans="2:8" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:8" ht="31.5" customHeight="1">
       <c r="B11" s="12">
         <v>8</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="D11" s="13"/>
       <c r="E11" s="13"/>
       <c r="F11" s="14" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G11" s="13"/>
       <c r="H11" s="15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
-    <row r="12" spans="2:8" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:8" ht="31.5" customHeight="1">
       <c r="B12" s="12">
         <v>9</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="D12" s="13"/>
       <c r="E12" s="13"/>
@@ -1454,24 +1465,24 @@
       </c>
       <c r="G12" s="13"/>
       <c r="H12" s="15" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
-    <row r="13" spans="2:8" ht="52.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:8" ht="52.5" customHeight="1" thickBot="1">
       <c r="B13" s="5">
         <v>10</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
       <c r="F13" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G13" s="1"/>
       <c r="H13" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>